<commit_message>
Add GitHub API Sync for Live database Updates
</commit_message>
<xml_diff>
--- a/data/IoT.xlsx
+++ b/data/IoT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6560a448ac85dd21/SKILLO/ProjectXYZ/PXYZ_APP/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="8_{8CD77BC7-6B55-4330-A131-D7E5F49AC3D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0BFD4379-2491-4597-B307-38F03372D1B4}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{8CD77BC7-6B55-4330-A131-D7E5F49AC3D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{747432CA-FF98-4B44-98BF-37DD8AE54D16}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7EC9D824-FD71-4C0A-A0F2-D44867FB9F29}"/>
+    <workbookView minimized="1" xWindow="7716" yWindow="5064" windowWidth="15324" windowHeight="7176" xr2:uid="{7EC9D824-FD71-4C0A-A0F2-D44867FB9F29}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -63773,7 +63773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="932" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
+    <row r="932" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A932" t="s">
         <v>1041</v>
       </c>
@@ -63826,7 +63826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="933" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
+    <row r="933" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A933" t="s">
         <v>1042</v>
       </c>
@@ -63879,7 +63879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="934" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
+    <row r="934" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A934" t="s">
         <v>1043</v>
       </c>
@@ -66635,7 +66635,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="986" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
+    <row r="986" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A986" t="s">
         <v>1098</v>
       </c>
@@ -66688,7 +66688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="987" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
+    <row r="987" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A987" t="s">
         <v>1099</v>
       </c>
@@ -66741,7 +66741,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="988" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
+    <row r="988" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A988" t="s">
         <v>1100</v>
       </c>
@@ -88154,7 +88154,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1310" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1310" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A1310" t="s">
         <v>1440</v>
       </c>
@@ -88207,7 +88207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1311" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1311" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A1311" t="s">
         <v>1441</v>
       </c>
@@ -88260,7 +88260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1312" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1312" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A1312" t="s">
         <v>1442</v>
       </c>
@@ -91016,7 +91016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1364" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1364" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A1364" t="s">
         <v>1497</v>
       </c>
@@ -91069,7 +91069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1365" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1365" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A1365" t="s">
         <v>1498</v>
       </c>
@@ -91122,7 +91122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1366" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1366" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A1366" t="s">
         <v>1499</v>
       </c>
@@ -97917,7 +97917,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="1474" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1474" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A1474" t="s">
         <v>1613</v>
       </c>
@@ -108800,7 +108800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1634" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1634" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A1634" t="s">
         <v>1782</v>
       </c>
@@ -108853,7 +108853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1635" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1635" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A1635" t="s">
         <v>1783</v>
       </c>
@@ -108906,7 +108906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1636" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1636" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A1636" t="s">
         <v>1784</v>
       </c>
@@ -111033,11 +111033,6 @@
         <filter val="IM5"/>
       </filters>
     </filterColumn>
-    <filterColumn colId="8">
-      <filters>
-        <filter val="ON"/>
-      </filters>
-    </filterColumn>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>